<commit_message>
FraSoHome Live fase 7: documentación del escenario 11
- README del escenario 11 con arquitectura, recursos, despliegue y guion de cada uno de los 16 escenarios
- Diagrama draw.io de la arquitectura (diagramas/arquitectura-web-transaccional)
- Escenario 11 en el catálogo de escenarios, el README raíz, el índice de diagramas y la matriz de recursos (CSV y Excel)
- Nota «Con datos vivos» en los escenarios 02 a 10, con la exportación marcada como pendiente (fase 5)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/escenarios/recursos-por-escenario.xlsx
+++ b/escenarios/recursos-por-escenario.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recursos por escenario" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catálogo de datos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Recursos por escenario" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Catálogo de datos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recursos por escenario'!$A$1:$F$124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Recursos por escenario'!$A$1:$F$141</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catálogo de datos'!$A$1:$H$74</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F124"/>
+  <dimension ref="A1:F141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -488,13 +488,11 @@
           <t>Visor de CSV o Excel</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -512,13 +510,11 @@
           <t>Proyector</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -536,13 +532,11 @@
           <t>Microsoft Fabric (Lakehouse + notebooks) o Python 3.10+ local</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -560,13 +554,11 @@
           <t>Streamlit (app)</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -584,13 +576,11 @@
           <t>Azure SQL Database o Fabric SQL Database</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -608,13 +598,11 @@
           <t>sqlcmd con autenticación Entra</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -632,13 +620,11 @@
           <t>Fabric CLI</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -656,13 +642,11 @@
           <t>PowerShell 7</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -680,13 +664,11 @@
           <t>Python + pyodbc (opcional)</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -704,13 +686,11 @@
           <t>Python 3.10+ con pandas, scikit-learn, shap, lime</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -728,13 +708,11 @@
           <t>Jupyter</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -752,13 +730,11 @@
           <t>Python 3.10+ con pandas, scikit-learn</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -776,13 +752,11 @@
           <t>Streamlit + Altair</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -800,13 +774,11 @@
           <t>Jupyter</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -824,13 +796,11 @@
           <t>Power BI Desktop o Service</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -848,13 +818,11 @@
           <t>ChatGPT/Copilot (opcional)</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -872,13 +840,11 @@
           <t>Copilot Studio</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -896,13 +862,11 @@
           <t>Entorno Power Platform con Dataverse</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -920,13 +884,11 @@
           <t>Capacidad Microsoft Fabric con IQ (preview)</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -944,13 +906,11 @@
           <t>PowerShell 7 + Azure CLI</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -968,13 +928,11 @@
           <t>Opciones de tenant Ontology, Graph y Data Agent</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -992,13 +950,11 @@
           <t>Python 3.10+ con pandas, scikit-learn, python-docx, pyarrow</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1016,13 +972,11 @@
           <t>Jupyter</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1040,13 +994,11 @@
           <t>Proyecto Microsoft Foundry con Agent Service</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1064,13 +1016,11 @@
           <t>Code Interpreter, File Search y búsqueda web</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1098,7 +1048,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1126,7 +1075,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1154,7 +1102,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1182,7 +1129,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1210,7 +1156,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1238,7 +1183,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1266,7 +1210,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1294,7 +1237,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1322,7 +1264,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1350,7 +1291,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1378,7 +1318,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1406,7 +1345,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1434,7 +1372,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1462,7 +1399,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1490,7 +1426,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1518,7 +1453,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1546,7 +1480,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1574,7 +1507,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1602,7 +1534,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1630,7 +1561,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1658,7 +1588,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1686,7 +1615,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1714,7 +1642,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1742,7 +1669,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1770,7 +1696,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1798,7 +1723,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1826,7 +1750,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1854,7 +1777,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1882,7 +1804,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1910,7 +1831,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1938,7 +1858,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1966,7 +1885,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1994,7 +1912,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2022,7 +1939,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2050,7 +1966,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2078,7 +1993,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2106,7 +2020,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2134,7 +2047,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2162,7 +2074,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2190,7 +2101,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2730,7 +2640,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2758,7 +2667,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2786,7 +2694,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2814,7 +2721,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2842,7 +2748,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2870,7 +2775,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2898,7 +2802,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2926,7 +2829,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2954,7 +2856,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2982,7 +2883,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3010,7 +2910,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3038,7 +2937,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3066,7 +2964,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3094,7 +2991,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3122,7 +3018,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3150,7 +3045,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3178,7 +3072,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3206,7 +3099,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3234,7 +3126,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3262,7 +3153,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3290,7 +3180,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3318,7 +3207,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -3346,7 +3234,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3374,7 +3261,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -3402,7 +3288,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3430,7 +3315,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3458,7 +3342,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3486,7 +3369,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3514,7 +3396,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3542,7 +3423,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3570,7 +3450,6 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3918,10 +3797,443 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="F124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>11 · Web transaccional (FraSoHome Live)</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Entorno</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Suscripción de Azure con permisos de propietario (servicios gratuitos)</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>11 · Web transaccional (FraSoHome Live)</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Entorno</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Azure CLI 2.53 o superior</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>11 · Web transaccional (FraSoHome Live)</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Entorno</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Python 3.10+ (los scripts preparan su entorno)</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>11 · Web transaccional (FraSoHome Live)</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Entorno</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Node.js (CLI de Static Web Apps)</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>11 · Web transaccional (FraSoHome Live)</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Entorno</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>PowerShell</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>11 · Web transaccional (FraSoHome Live)</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Entorno</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>GitHub CLI y entorno de GitHub Actions</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Publicación automática</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>11 · Web transaccional (FraSoHome Live)</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Entorno</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Navegador actual</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>11 · Web transaccional (FraSoHome Live)</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Los 64 CSV de datos/</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>datos/</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>58 se cargan en SQL y Cosmos; 6 se recalculan al exportar</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>11 · Web transaccional (FraSoHome Live)</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Ficha y guiones de los 16 escenarios</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>escenarios/11-web-transaccional/README.md</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>11 · Web transaccional (FraSoHome Live)</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Cómo está hecha la web</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>escenarios/11-web-transaccional/web.md</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>11 · Web transaccional (FraSoHome Live)</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>app/ (web)</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>escenarios/11-web-transaccional/app/</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>11 · Web transaccional (FraSoHome Live)</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>api/ (143 endpoints)</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>escenarios/11-web-transaccional/api/</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>11 · Web transaccional (FraSoHome Live)</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>sql/ (modelo y procedimientos)</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>escenarios/11-web-transaccional/sql/</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>11 · Web transaccional (FraSoHome Live)</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>seed/ (carga inicial y reinicio)</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>escenarios/11-web-transaccional/seed/</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>11 · Web transaccional (FraSoHome Live)</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>infra/ (Bicep y GitHub Actions)</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>escenarios/11-web-transaccional/infra/</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>11 · Web transaccional (FraSoHome Live)</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>tools/ (usuarios, configuración y publicación)</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>escenarios/11-web-transaccional/tools/</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>11 · Web transaccional (FraSoHome Live)</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>arquitectura-web-transaccional.drawio.svg</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>diagramas/arquitectura-web-transaccional.drawio.svg</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F124"/>
+  <autoFilter ref="A1:F141"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5419,8 +5731,6 @@
           <t>Documento</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>01, 03, 07, 09</t>
@@ -5453,8 +5763,6 @@
           <t>Documento</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>01, 03, 07, 09</t>
@@ -5487,8 +5795,6 @@
           <t>Documento</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>01, 03, 07, 09</t>
@@ -5521,8 +5827,6 @@
           <t>Documento</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>01, 03, 07, 09</t>
@@ -5555,8 +5859,6 @@
           <t>Documento</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>01, 03, 07, 09</t>
@@ -5589,8 +5891,6 @@
           <t>Documento</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>01, 03, 07, 09</t>
@@ -5623,8 +5923,6 @@
           <t>Documento</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>01, 03, 07, 09</t>
@@ -5657,8 +5955,6 @@
           <t>Documento</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>01, 03, 07, 09</t>
@@ -5691,8 +5987,6 @@
           <t>Documento</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>01, 03, 07, 09</t>
@@ -5725,8 +6019,6 @@
           <t>Documento</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>01, 03, 07, 09</t>

</xml_diff>